<commit_message>
gop cac cell trong ModelComparision lai cho gon, bo sung notebook test cach lam cua Entropy
</commit_message>
<xml_diff>
--- a/notebooks/Model_Comparison/results/model_comparison/error_analysis_summary.xlsx
+++ b/notebooks/Model_Comparison/results/model_comparison/error_analysis_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,25 +436,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MAPE (%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>R2 Score</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Mean Error</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Median Error</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Max Error</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Top 10 Errors</t>
         </is>
@@ -467,18 +477,24 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>141614.9019710154</v>
+      </c>
+      <c r="C2" t="n">
+        <v>131.3166693038851</v>
+      </c>
+      <c r="D2" t="n">
         <v>0.1533230485853148</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>19781.58634313867</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>2172.368029226232</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>10133570.77990773</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>10,133,571, 3,552,596, 3,229,319, 2,560,442, 2,470,909, 1,597,745, 1,526,178, 1,449,783, 1,412,487, 1,371,568</t>
         </is>
@@ -491,18 +507,24 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>147166.508588011</v>
+      </c>
+      <c r="C3" t="n">
+        <v>124.3983461283009</v>
+      </c>
+      <c r="D3" t="n">
         <v>0.08563877949847076</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>19866.5865045202</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>2437.34765625</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>10130114.2421875</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>10,130,114, 5,367,037, 3,539,316, 2,562,890, 2,468,884, 1,598,467, 1,444,556, 1,328,721, 1,269,245, 1,250,376</t>
         </is>
@@ -515,18 +537,24 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>150822.7482342702</v>
+      </c>
+      <c r="C4" t="n">
+        <v>153.7810182872185</v>
+      </c>
+      <c r="D4" t="n">
         <v>0.03964118864003152</v>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>20568.20169733818</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>2677.28487942866</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>10125644.90130663</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>10,125,645, 5,977,706, 3,537,683, 2,552,923, 2,462,302, 1,597,842, 1,542,371, 1,447,186, 1,382,346, 1,251,703</t>
         </is>
@@ -539,18 +567,24 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>152039.4693290611</v>
+      </c>
+      <c r="C5" t="n">
+        <v>161.0958018710449</v>
+      </c>
+      <c r="D5" t="n">
         <v>0.02408382651256213</v>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>21643.49842965811</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>3031.913895542814</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>10140715.79560063</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>10,140,716, 6,010,706, 3,547,939, 2,549,190, 2,476,004, 1,596,513, 1,575,063, 1,447,695, 1,443,233, 1,340,971</t>
         </is>
@@ -563,18 +597,24 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>155254.015657576</v>
+      </c>
+      <c r="C6" t="n">
+        <v>173.8979858588901</v>
+      </c>
+      <c r="D6" t="n">
         <v>-0.01761970827448023</v>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>23985.88273812434</v>
       </c>
-      <c r="D6" t="n">
+      <c r="F6" t="n">
         <v>3583.913750575518</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>10141075.37658731</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>10,141,075, 6,011,666, 3,555,244, 2,564,427, 2,469,253, 1,765,281, 1,595,166, 1,447,885, 1,285,781, 1,244,880</t>
         </is>
@@ -587,18 +627,24 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>155259.3739211261</v>
+      </c>
+      <c r="C7" t="n">
+        <v>173.8628126187824</v>
+      </c>
+      <c r="D7" t="n">
         <v>-0.01768995146479524</v>
       </c>
-      <c r="C7" t="n">
+      <c r="E7" t="n">
         <v>23987.2860304637</v>
       </c>
-      <c r="D7" t="n">
+      <c r="F7" t="n">
         <v>3588.662968863008</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>10141044.75702388</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>10,141,045, 6,011,640, 3,555,234, 2,564,436, 2,469,233, 1,765,088, 1,595,167, 1,447,885, 1,285,819, 1,244,884</t>
         </is>
@@ -611,18 +657,24 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>155353.4424325848</v>
+      </c>
+      <c r="C8" t="n">
+        <v>204.4470970070549</v>
+      </c>
+      <c r="D8" t="n">
         <v>-0.01892352052614021</v>
       </c>
-      <c r="C8" t="n">
+      <c r="E8" t="n">
         <v>25793.8137868117</v>
       </c>
-      <c r="D8" t="n">
+      <c r="F8" t="n">
         <v>5287.700517037335</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>10164122.29948296</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>10,164,122, 6,027,122, 3,566,122, 2,568,122, 2,491,122, 1,842,122, 1,592,122, 1,574,192, 1,461,122, 1,392,122</t>
         </is>
@@ -635,18 +687,24 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>155353.4424325848</v>
+      </c>
+      <c r="C9" t="n">
+        <v>204.4470970070549</v>
+      </c>
+      <c r="D9" t="n">
         <v>-0.01892352052614021</v>
       </c>
-      <c r="C9" t="n">
+      <c r="E9" t="n">
         <v>25793.8137868117</v>
       </c>
-      <c r="D9" t="n">
+      <c r="F9" t="n">
         <v>5287.700517037335</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>10164122.29948296</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>10,164,122, 6,027,122, 3,566,122, 2,568,122, 2,491,122, 1,842,122, 1,592,122, 1,574,192, 1,461,122, 1,392,122</t>
         </is>

</xml_diff>